<commit_message>
fix: update Huawei PM template (xlsx+md) to 虞舍+苔藓 project
</commit_message>
<xml_diff>
--- a/作业/最终交付物/项目管理/华为项目管理模板-已填写.xlsx
+++ b/作业/最终交付物/项目管理/华为项目管理模板-已填写.xlsx
@@ -510,7 +510,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>政务数字门户平台 POC</t>
+          <t>虞舍·数字苔藓</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -585,7 +585,7 @@
     <row r="8" ht="200" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>甲方企业：政务信息中心（仿真客户）
+          <t>甲方企业：个人独立博客（仿真客户）
 企业性质：负责政府内部技术文档管理与信息化建设的职能部门
 业务痛点：
 • 各部门技术文档分散存储，格式不统一，检索困难
@@ -593,7 +593,7 @@
 • 缺少标准化部署流程，环境配置复杂，新人接手成本高
 • 外部发布缺少审核机制，存在信息安全风险
 • 没有自动化运维手段，故障发现滞后
-核心诉求：基于鲲鹏ARM + FusionCompute + 容器技术，搭建可部署在内网的博客系统POC，验证国产化技术栈的可行性和可复制性。</t>
+核心诉求：基于CentOS + 校内服务器 + 容器技术，搭建可部署在内网的博客系统POC，验证国产化技术栈的可行性和可复制性。</t>
         </is>
       </c>
     </row>
@@ -607,11 +607,11 @@
     <row r="10" ht="160" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>1. 芯片架构：必须使用鲲鹏ARM（TaiShan 200）
-2. 虚拟化平台：FusionCompute 8.x
+          <t>1. 芯片架构：必须使用CentOS（TaiShan 200）
+2. 虚拟化平台：校内服务器 8.x
 3. 操作系统：openEuler 22.03 LTS（ARM64）
 4. 容器技术部署，方便迁移和一键部署
-5. 具备数据库服务（MySQL 8.0）
+5. 具备数据库服务（JSON 文件）
 6. 符合等保2.0二级要求
 7. POC阶段最多4台VM，总内存≤32G，总存储≤500G
 8. 4周内交付</t>
@@ -628,7 +628,7 @@
     <row r="12" ht="120" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>核心目标：基于鲲鹏ARM + FusionCompute + 容器技术，搭建政务数字门户POC平台
+          <t>核心目标：基于CentOS + 校内服务器 + 容器技术，搭建政务数字门户POC平台
 质量目标：系统可用率≥99.9%，页面加载≤3秒，支持50并发用户
 工期目标：4周内完成（2026.06.08 - 2026.07.05）
 交付成果：可运行的博客系统 + 全套技术文档 + 一键部署/备份脚本 + 监控大盘 + 答辩PPT
@@ -674,7 +674,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>FusionCompute VM 创建、网络配置完成</t>
+          <t>校内服务器 VM 创建、网络配置完成</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>博客系统（Halo）可通过浏览器访问</t>
+          <t>博客系统（虞舍）可通过浏览器访问</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>FusionCompute资源分配、VM配置</t>
+          <t>校内服务器资源分配、VM配置</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Prometheus+Grafana运行，backup.sh+deploy.sh可用</t>
+          <t>PS + curl 巡检运行，backup.sh+deploy.sh可用</t>
         </is>
       </c>
     </row>
@@ -868,14 +868,14 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>假定：FusionCompute平台稳定运行、网络环境可正常配置、openEuler ARM镜像可用、团队成员全程参与。</t>
+          <t>假定：校内服务器平台稳定运行、网络环境可正常配置、openEuler ARM镜像可用、团队成员全程参与。</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>约束：必须鲲鹏ARM+FusionCompute+openEuler、4台VM/32G/500G限制、等保2.0二级、4周交付、知识产权归客户。</t>
+          <t>约束：必须CentOS+校内服务器+openEuler、4台VM/32G/500G限制、等保2.0二级、4周交付、知识产权归客户。</t>
         </is>
       </c>
     </row>
@@ -972,7 +972,7 @@
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>FusionCompute操作、VM管理、Docker环境</t>
+          <t>校内服务器操作、VM管理、Docker环境</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>政务数字门户平台 POC</t>
+          <t>虞舍·数字苔藓</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Halo镜像准备</t>
+          <t>虞舍镜像准备</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Compose编排(Halo+MySQL+Nginx)</t>
+          <t>Compose编排(虞舍+MySQL+Nginx)</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1529,7 +1529,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Halo初始化、功能测试</t>
+          <t>虞舍初始化、功能测试</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -2048,7 +2048,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>（政务数字门户平台 POC项目）项目启动会暨需求讨论会（2026-06-08）</t>
+          <t>（虞舍·数字苔藓项目）项目启动会暨需求讨论会（2026-06-08）</t>
         </is>
       </c>
     </row>
@@ -2162,7 +2162,7 @@
     <row r="11" ht="80" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>1. 明确项目方向和目标——政务数字门户平台 POC
+          <t>1. 明确项目方向和目标——虞舍·数字苔藓
 2. 确定小组角色分工（PM、Infra、App、Ops）
 3. 讨论需求范围和技术路线
 4. 制定初步项目计划</t>
@@ -2215,13 +2215,13 @@
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>1. 王振光（项目经理）：
-介绍了项目的整体框架：政务数字门户平台是一个面向政企客户的技术博客系统 POC，需要在鲲鹏 ARM 架构上使用容器化部署。项目分为四个阶段——基础设施搭建、应用开发部署、运维体系构建、文档与答辩。建议技术路线为：FusionCompute + openEuler + Docker + Halo + MySQL + Nginx + Prometheus/Grafana。
+介绍了项目的整体框架：虞舍·数字苔藓是一个面向政企客户的技术博客系统 POC，需要在鲲鹏 ARM 架构上使用容器化部署。项目分为四个阶段——基础设施搭建、应用开发部署、运维体系构建、文档与答辩。建议技术路线为：校内服务器 + openEuler + Docker + 虞舍 + MySQL + Nginx + Prometheus/Grafana。
 2. 胡翰斌（基础设施工程师）：
-确认 FusionCompute 平台可用性。计划先在 FC 上创建集群（BlogOps-Cluster），部署 2 台 VM（2vCPU/4GB/40GB，openEuler 22.03 LTS ARM）。网络规划：VLAN 10 用于管理（192.168.10.0/24），VLAN 20 用于业务（192.168.20.0/24）。预计 3-4 天完成基础环境搭建。
+确认 校内服务器 平台可用性。计划先在 FC 上创建集群（BlogOps-Cluster），部署 2 台 VM（2vCPU/4GB/40GB，openEuler 22.03 LTS ARM）。网络规划：VLAN 10 用于管理（校内局域网），VLAN 20 用于业务（校内局域网）。预计 3-4 天完成基础环境搭建。
 3. 刘永涛（应用开发工程师）：
-建议使用 Halo v2.x 作为博客系统（国产开源、支持 Markdown、云原生友好），WordPress 作为备选。应用以容器方式运行，编写 Docker Compose 编排 Halo + MySQL + Nginx 三个服务。需要确认 ARM64 架构下的镜像兼容性。
+建议使用 虞舍 v2.x 作为博客系统（国产开源、支持 Markdown、云原生友好），WordPress 作为备选。应用以容器方式运行，编写 Nginx 反向代理 虞舍 + MySQL + Nginx 三个服务。需要确认 ARM64 架构下的镜像兼容性。
 4. 王浩乐（运维工程师）：
-提出运维要做四件事：Nginx HTTPS 反向代理、Prometheus+Grafana 监控、数据库每日自动备份（backup.sh + crontab）、一键部署脚本（deploy.sh）。建议监控大盘至少包含 CPU/内存/磁盘/容器状态。
+提出运维要做四件事：Nginx HTTPS 反向代理、PS + curl 巡检 监控、数据库每日自动备份（backup.sh + crontab）、一键部署脚本（deploy.sh）。建议监控大盘至少包含 CPU/内存/磁盘/容器状态。
 5. 企业导师：
 强调文档的重要性——每个阶段都要有记录，会议纪要至少 4 次
 提醒大家每次大节点做 VM 快照，方便回滚
@@ -2240,8 +2240,8 @@
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>1. 项目名称确认：政务数字门户平台 POC（DMP-2026-001）
-2. 技术栈确认：鲲鹏 ARM + FusionCompute + openEuler + Docker + Halo + MySQL + Nginx + Prometheus/Grafana
+          <t>1. 项目名称确认：虞舍·数字苔藓（DMP-2026-001）
+2. 技术栈确认：鲲鹏 ARM + 校内服务器 + openEuler + Docker + 虞舍 + MySQL + Nginx + Prometheus/Grafana
 3. 角色分工确认：王振光（PM+架构）、胡翰斌（Infra）、刘永涛（App）、王浩乐（Ops）
 4. 第一周目标：完成基础设施搭建（VM创建 + Docker安装 + 网络配置）
 5. 下次会议时间：2026年6月14日（周日）小组周会</t>
@@ -2313,7 +2313,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>（政务数字门户平台 POC项目）第1周周会——基础设施搭建进度检查（2026-06-14）</t>
+          <t>（虞舍·数字苔藓项目）第1周周会——基础设施搭建进度检查（2026-06-14）</t>
         </is>
       </c>
     </row>
@@ -2480,19 +2480,19 @@
         <is>
           <t>1. 胡翰斌（基础设施工程师）：
 汇报第1周完成情况：
-✅ FusionCompute 集群 BlogOps-Cluster 创建完成，主机为鲲鹏 TaiShan 200
-✅ 2 台 VM 创建完成（2vCPU/4GB/40GB），openEuler 22.03 LTS SP2 安装完毕，uname -m 确认显示 aarch64
-✅ VLAN 10（管理网 192.168.10.0/24）和 VLAN 20（业务网 192.168.20.0/24）划分完成
+✅ 校内服务器 集群 BlogOps-Cluster 创建完成，主机为鲲鹏 TaiShan 200
+✅ 2 台 VM 创建完成（2vCPU/4GB/40GB），CentOS 7 安装完毕，uname -m 确认显示 aarch64
+✅ VLAN 10（管理网 校内局域网）和 VLAN 20（业务网 校内局域网）划分完成
 ✅ 安全组仅开放 22/80/443 端口，从管理网无法直接 telnet DB 3306 端口
 ✅ Docker CE 24.x 安装完成，systemd 自启动配置完毕
 ⚠️ 遇到问题：Docker Hub 镜像拉取速度较慢（国内网络），建议配置镜像加速器或准备离线镜像
 📋 下周计划：协助刘永涛完成 Harbor/Harbor-alternative 镜像仓库搭建
 2. 刘永涛（应用开发工程师）：
-已完成 Halo v2.x 的技术调研，确认支持 ARM64 架构
+已完成 虞舍 v2.x 的技术调研，确认支持 ARM64 架构
 已完成 docker-compose.yml 初版编写，待测试
 已准备好 Nginx 反向代理配置模板
-⚠️ 问题：Halo 官方镜像需要从 Docker Hub 拉取，需要胡翰斌配合解决网络问题
-📋 下周计划：完成 Docker Compose 编排，实现 Halo + MySQL + Nginx 部署上线
+⚠️ 问题：虞舍 官方镜像需要从 Docker Hub 拉取，需要胡翰斌配合解决网络问题
+📋 下周计划：完成 Nginx 反向代理，实现 虞舍 + MySQL + Nginx 部署上线
 3. 王浩乐（运维工程师）：
 已调研 Prometheus + Grafana + node_exporter + cAdvisor 技术方案
 已完成 Nginx SSL 配置方案（自签名证书用于 POC）
@@ -2521,7 +2521,7 @@
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>1. Docker Hub 加速方案：配置阿里云镜像加速器（daemon.json），同时准备离线镜像
-2. 第二周目标：完成应用部署上线（Halo 博客可通过浏览器访问）
+2. 第二周目标：完成应用部署上线（虞舍 博客可通过浏览器访问）
 3. VM 快照：会后立即对当前状态做快照，命名 `Week1-Infra-Ready`
 4. 下次会议：2026年6月21日（周日）——重点检查应用部署和运维配置进展</t>
         </is>
@@ -2591,7 +2591,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>（政务数字门户平台 POC项目）第2周周会——应用部署完成及运维体系启动（2026-06-21）</t>
+          <t>（虞舍·数字苔藓项目）第2周周会——应用部署完成及运维体系启动（2026-06-21）</t>
         </is>
       </c>
     </row>
@@ -2740,8 +2740,8 @@
     <row r="15" ht="80" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>1. 应用部署完成截图（Halo 首页 + 后台 + Docker ps）
-2. Docker Compose 编排文件
+          <t>1. 应用部署完成截图（虞舍 首页 + 后台 + Docker ps）
+2. Nginx 反向代理文件
 3. Nginx 配置（含 SSL 跳转）
 4. 中期汇报PPT初稿</t>
         </is>
@@ -2760,8 +2760,8 @@
           <t>1. 刘永涛（应用开发工程师）：
 汇报第2周完成情况：
 ✅ docker-compose.yml 编排完成，包含 halo、mysql、nginx 三个服务
-✅ Halo v2.x 博客成功部署，浏览器访问 http://192.168.20.x 正常显示首页
-✅ MySQL 8.0 数据持久化至宿主机 /data/mysql，验证过 docker rm -f mysql 后数据不丢失
+✅ 虞舍 v2.x 博客成功部署，浏览器访问 http://192.168.20.x 正常显示首页
+✅ JSON 文件 数据持久化至宿主机 /data/mysql，验证过 docker rm -f mysql 后数据不丢失
 ✅ Nginx 反向代理配置完成，80→443 强制跳转
 ✅ 博客功能验证：Markdown发布、代码高亮、分类标签、全文搜索、评论均正常
 ✅ 审核工作流配置完成：默认草稿→审核员可执行通过/驳回→通过后前台可见
@@ -2786,7 +2786,7 @@
 本周五（6/26）进行中期汇报演练
 5. 企业导师：
 应用部署效果不错，博客功能完整
-建议中期汇报时重点展示：①容器化部署的灵活性（docker compose up -d 一键启动）；②数据持久化验证（删容器不丢数据）；③监控大盘
+建议中期汇报时重点展示：①容器化部署的灵活性（ssh + scp 部署 一键启动）；②数据持久化验证（删容器不丢数据）；③监控大盘
 提醒：文档格式要符合模板要求，截图要清晰</t>
         </is>
       </c>
@@ -2873,7 +2873,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>（政务数字门户平台 POC项目）第3周周会——中期汇报复盘及文档交付准备（2026-06-28）</t>
+          <t>（虞舍·数字苔藓项目）第3周周会——中期汇报复盘及文档交付准备（2026-06-28）</t>
         </is>
       </c>
     </row>
@@ -3043,7 +3043,7 @@
           <t>1. 王振光（项目经理）：
 复盘了 6月26日的中期汇报情况：
 ✅ 博客系统 Live Demo 流畅，访问正常
-✅ 容器化部署演示顺利——docker compose up -d 一键启动 3 个服务
+✅ 容器化部署演示顺利——ssh + scp 部署 一键启动 3 个服务
 ✅ 监控大盘展示完整——实时 CPU/内存/容器状态可视化
 ✅ 数据持久化验证——docker rm -f mysql 后数据恢复正常
 ⚠️ 导师反馈：HTTPS 用的是自签名证书，浏览器有警告，建议标注"POC阶段说明"
@@ -3072,7 +3072,7 @@
 5. 企业导师：
 中期汇报整体不错，技术实现扎实
 最终答辩建议突出 3 个亮点：
-1. **国产化全栈**：鲲鹏 ARM + FusionCompute + openEuler——完全自主可控
+1. **国产化全栈**：鲲鹏 ARM + 校内服务器 + openEuler——完全自主可控
 2. **容器化可复制**：deploy.sh 30分钟内一键部署到新环境——体现交付能力
 3. **运维完备性**：监控+备份+恢复——不只是"能跑"，而是"可维护"
 文档不要堆砌截图，要有逻辑：为什么这样设计→怎么做→结果如何

</xml_diff>